<commit_message>
reformatting and cleaning up
</commit_message>
<xml_diff>
--- a/Dependencies/Takasugi_2024/PTM_heatmap_df.xlsx
+++ b/Dependencies/Takasugi_2024/PTM_heatmap_df.xlsx
@@ -958,7 +958,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Acetaldehyde +28</t>
+          <t>Ethylation</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -983,7 +983,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
@@ -1110,7 +1110,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Ethylation</t>
+          <t>Acetaldehyde +28</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1135,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -3314,7 +3314,7 @@
     <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
-          <t>ubiquitinylation residue</t>
+          <t>Double Carbamidomethylation</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -3390,7 +3390,7 @@
     <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
-          <t>Double Carbamidomethylation</t>
+          <t>ubiquitinylation residue</t>
         </is>
       </c>
       <c r="B40" t="n">

</xml_diff>